<commit_message>
Update techno funda screener data
</commit_message>
<xml_diff>
--- a/data/techno-funda-trade-sheet.xlsx
+++ b/data/techno-funda-trade-sheet.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="53">
   <si>
     <t>Metric</t>
   </si>
@@ -25,7 +25,7 @@
     <t>Updated At</t>
   </si>
   <si>
-    <t>2026-07-07T04:54:55.494Z</t>
+    <t>2026-07-07T18:44:43.240Z</t>
   </si>
   <si>
     <t>Open Trades</t>
@@ -79,10 +79,100 @@
     <t>Holding Days</t>
   </si>
   <si>
+    <t>Setup Score</t>
+  </si>
+  <si>
+    <t>Sector Breadth</t>
+  </si>
+  <si>
+    <t>Near 52W High</t>
+  </si>
+  <si>
+    <t>55D Breakout</t>
+  </si>
+  <si>
+    <t>Volume Ratio</t>
+  </si>
+  <si>
+    <t>Risk To ST %</t>
+  </si>
+  <si>
+    <t>Previous Low</t>
+  </si>
+  <si>
+    <t>2 Candle Low</t>
+  </si>
+  <si>
+    <t>4 Candle Low</t>
+  </si>
+  <si>
     <t>Entry Reason</t>
   </si>
   <si>
     <t>Exit Reason</t>
+  </si>
+  <si>
+    <t>Default Nifty 500</t>
+  </si>
+  <si>
+    <t>CUB</t>
+  </si>
+  <si>
+    <t>City Union Bank Ltd.</t>
+  </si>
+  <si>
+    <t>OPEN</t>
+  </si>
+  <si>
+    <t>2026-07-06</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>41.58% (42/101)</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Weekly RSI 64.23 is above 50. Daily RSI 73.78 is above 50. Weekly RS 4.9% is above 0. Daily long RS55 10.0% is above 0. Daily short RS21 17.3% is above 0. Daily close 224.69 is above Supertrend(10, 3) 198.54. Price action strength: close crossed 55-day high 220.24. RS trend strength: weekly RS and daily RS55 are rising. Trend strength: close is above 50-DMA and 200-DMA, with fast DMA above slow DMA.</t>
+  </si>
+  <si>
+    <t>SHREECEM</t>
+  </si>
+  <si>
+    <t>Shree Cement Ltd.</t>
+  </si>
+  <si>
+    <t>18.18% (2/11)</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Weekly RSI 55.89 is above 50. Daily RSI 65.39 is above 50. Weekly RS 1.4% is above 0. Daily long RS55 1.9% is above 0. Daily short RS21 6.0% is above 0. Daily close 26630.00 is above Supertrend(10, 3) 25006.27. RS trend strength: weekly RS and daily RS55 are rising. Risk reference: close is 6.10% above daily Supertrend.</t>
+  </si>
+  <si>
+    <t>CANFINHOME</t>
+  </si>
+  <si>
+    <t>Can Fin Homes Ltd.</t>
+  </si>
+  <si>
+    <t>Weekly RSI 60.24 is above 50. Daily RSI 66.02 is above 50. Weekly RS 3.4% is above 0. Daily long RS55 3.0% is above 0. Daily short RS21 9.0% is above 0. Daily close 918.80 is above Supertrend(10, 3) 836.75. Price action strength: close is within 15% of 52-week high 971.50. RS trend strength: weekly RS and daily RS55 are rising.</t>
+  </si>
+  <si>
+    <t>CONCORDBIO</t>
+  </si>
+  <si>
+    <t>Concord Biotech Ltd.</t>
+  </si>
+  <si>
+    <t>61.22% (30/49)</t>
+  </si>
+  <si>
+    <t>Weekly RSI 52.76 is above 50. Daily RSI 53.60 is above 50. Weekly RS 7.8% is above 0. Daily long RS55 17.4% is above 0. Daily short RS21 1.7% is above 0. Daily close 1283.60 is above Supertrend(10, 3) 1205.14. RS trend strength: weekly RS and daily RS55 are rising. Risk reference: close is 6.11% above daily Supertrend. Sector breadth strong: Healthcare has 30/49 stocks (61.22%) passing daily strength.</t>
   </si>
 </sst>
 </file>
@@ -497,7 +587,7 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -532,7 +622,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -544,11 +634,13 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="15" width="54" customWidth="1"/>
+    <col min="13" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="22" width="14" customWidth="1"/>
+    <col min="23" max="24" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -594,9 +686,332 @@
       <c r="O1" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2">
+        <v>224.69</v>
+      </c>
+      <c r="G2">
+        <v>445</v>
+      </c>
+      <c r="H2">
+        <v>99987.05</v>
+      </c>
+      <c r="I2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2">
+        <v>8</v>
+      </c>
+      <c r="O2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>39</v>
+      </c>
+      <c r="R2">
+        <v>0.83</v>
+      </c>
+      <c r="S2">
+        <v>11.64</v>
+      </c>
+      <c r="T2">
+        <v>215.67</v>
+      </c>
+      <c r="U2">
+        <v>214.53</v>
+      </c>
+      <c r="V2">
+        <v>202.5</v>
+      </c>
+      <c r="W2" t="s">
+        <v>40</v>
+      </c>
+      <c r="X2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3">
+        <v>26630</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>79890</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3">
+        <v>6</v>
+      </c>
+      <c r="O3" t="s">
+        <v>43</v>
+      </c>
+      <c r="P3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>44</v>
+      </c>
+      <c r="R3">
+        <v>0.27</v>
+      </c>
+      <c r="S3">
+        <v>6.1</v>
+      </c>
+      <c r="T3">
+        <v>26345</v>
+      </c>
+      <c r="U3">
+        <v>25965</v>
+      </c>
+      <c r="V3">
+        <v>25055</v>
+      </c>
+      <c r="W3" t="s">
+        <v>45</v>
+      </c>
+      <c r="X3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4">
+        <v>918.8</v>
+      </c>
+      <c r="G4">
+        <v>108</v>
+      </c>
+      <c r="H4">
+        <v>99230.4</v>
+      </c>
+      <c r="I4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4">
+        <v>6</v>
+      </c>
+      <c r="O4" t="s">
+        <v>38</v>
+      </c>
+      <c r="P4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>44</v>
+      </c>
+      <c r="R4">
+        <v>1.23</v>
+      </c>
+      <c r="S4">
+        <v>8.93</v>
+      </c>
+      <c r="T4">
+        <v>879.1</v>
+      </c>
+      <c r="U4">
+        <v>878.3</v>
+      </c>
+      <c r="V4">
+        <v>845.65</v>
+      </c>
+      <c r="W4" t="s">
+        <v>48</v>
+      </c>
+      <c r="X4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5">
+        <v>1283.6</v>
+      </c>
+      <c r="G5">
+        <v>77</v>
+      </c>
+      <c r="H5">
+        <v>98837.2</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5">
+        <v>5</v>
+      </c>
+      <c r="O5" t="s">
+        <v>51</v>
+      </c>
+      <c r="P5" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>44</v>
+      </c>
+      <c r="R5">
+        <v>0.24</v>
+      </c>
+      <c r="S5">
+        <v>6.11</v>
+      </c>
+      <c r="T5">
+        <v>1260</v>
+      </c>
+      <c r="U5">
+        <v>1260</v>
+      </c>
+      <c r="V5">
+        <v>1260</v>
+      </c>
+      <c r="W5" t="s">
+        <v>52</v>
+      </c>
+      <c r="X5" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:X1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -604,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -616,11 +1031,13 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="15" width="54" customWidth="1"/>
+    <col min="13" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="22" width="14" customWidth="1"/>
+    <col min="23" max="24" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -666,9 +1083,332 @@
       <c r="O1" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2">
+        <v>224.69</v>
+      </c>
+      <c r="G2">
+        <v>445</v>
+      </c>
+      <c r="H2">
+        <v>99987.05</v>
+      </c>
+      <c r="I2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2">
+        <v>8</v>
+      </c>
+      <c r="O2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>39</v>
+      </c>
+      <c r="R2">
+        <v>0.83</v>
+      </c>
+      <c r="S2">
+        <v>11.64</v>
+      </c>
+      <c r="T2">
+        <v>215.67</v>
+      </c>
+      <c r="U2">
+        <v>214.53</v>
+      </c>
+      <c r="V2">
+        <v>202.5</v>
+      </c>
+      <c r="W2" t="s">
+        <v>40</v>
+      </c>
+      <c r="X2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3">
+        <v>26630</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>79890</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3">
+        <v>6</v>
+      </c>
+      <c r="O3" t="s">
+        <v>43</v>
+      </c>
+      <c r="P3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>44</v>
+      </c>
+      <c r="R3">
+        <v>0.27</v>
+      </c>
+      <c r="S3">
+        <v>6.1</v>
+      </c>
+      <c r="T3">
+        <v>26345</v>
+      </c>
+      <c r="U3">
+        <v>25965</v>
+      </c>
+      <c r="V3">
+        <v>25055</v>
+      </c>
+      <c r="W3" t="s">
+        <v>45</v>
+      </c>
+      <c r="X3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4">
+        <v>918.8</v>
+      </c>
+      <c r="G4">
+        <v>108</v>
+      </c>
+      <c r="H4">
+        <v>99230.4</v>
+      </c>
+      <c r="I4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4">
+        <v>6</v>
+      </c>
+      <c r="O4" t="s">
+        <v>38</v>
+      </c>
+      <c r="P4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>44</v>
+      </c>
+      <c r="R4">
+        <v>1.23</v>
+      </c>
+      <c r="S4">
+        <v>8.93</v>
+      </c>
+      <c r="T4">
+        <v>879.1</v>
+      </c>
+      <c r="U4">
+        <v>878.3</v>
+      </c>
+      <c r="V4">
+        <v>845.65</v>
+      </c>
+      <c r="W4" t="s">
+        <v>48</v>
+      </c>
+      <c r="X4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5">
+        <v>1283.6</v>
+      </c>
+      <c r="G5">
+        <v>77</v>
+      </c>
+      <c r="H5">
+        <v>98837.2</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5">
+        <v>5</v>
+      </c>
+      <c r="O5" t="s">
+        <v>51</v>
+      </c>
+      <c r="P5" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>44</v>
+      </c>
+      <c r="R5">
+        <v>0.24</v>
+      </c>
+      <c r="S5">
+        <v>6.11</v>
+      </c>
+      <c r="T5">
+        <v>1260</v>
+      </c>
+      <c r="U5">
+        <v>1260</v>
+      </c>
+      <c r="V5">
+        <v>1260</v>
+      </c>
+      <c r="W5" t="s">
+        <v>52</v>
+      </c>
+      <c r="X5" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:X1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -676,7 +1416,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -688,11 +1428,13 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="15" width="54" customWidth="1"/>
+    <col min="13" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="22" width="14" customWidth="1"/>
+    <col min="23" max="24" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -738,9 +1480,36 @@
       <c r="O1" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:X1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>